<commit_message>
Regenerate review package with anchoring instructions
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AzLhnR3PoLPQ3QmU5BGcpZ
</commit_message>
<xml_diff>
--- a/reports/review/top50_terms.xlsx
+++ b/reports/review/top50_terms.xlsx
@@ -195,7 +195,7 @@
     </comment>
     <comment ref="I1" authorId="0" shapeId="0">
       <text>
-        <t>Opcional: dúvidas, termo alternativo, uso regional.</t>
+        <t>Opcional: dúvidas, termo alternativo, uso regional. Se mantiver a candidata sem mudar nada, escreva: candidata aceita sem alteração</t>
       </text>
     </comment>
   </commentList>
@@ -491,7 +491,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D19"/>
+  <dimension ref="A1:D20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -525,178 +525,190 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>candidate_pt</t>
+          <t>Corrija sem receio</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>TRADUÇÃO AUTOMÁTICA (gerada por máquina). Exige revisão humana; não usar sem revisão. Fundo laranja. Vazia nesta versão: a variável ANTHROPIC_API_KEY não estava definida. A revisão pode ser feita direto em reviewer_pt.</t>
+          <t>A tradução candidata é só um ponto de partida e pode estar errada ou soar estranha. Corrija sem receio sempre que preferir outro termo. Se aceitar a candidata exatamente como está, copie-a em reviewer_pt e escreva em reviewer_notes: candidata aceita sem alteração. Isso permite medir quanto a tradução automática acertou.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Convenções</t>
+          <t>candidate_pt</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Grafia brasileira; termo usual na clínica e na genética médica no Brasil; forma de rótulo do HPO (substantivo, só a primeira letra maiúscula, sem ponto final).</t>
+          <t>TRADUÇÃO AUTOMÁTICA (gerada por máquina). Exige revisão humana; não usar sem revisão. Fundo laranja. Vazia nesta versão: a variável ANTHROPIC_API_KEY não estava definida. A revisão pode ser feita direto em reviewer_pt.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>label_en / definition_en / synonyms_en</t>
+          <t>Convenções</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>Rótulo, definição e sinônimos oficiais em inglês (HPO). Sinônimos que não são exatos aparecem marcados, por exemplo [related].</t>
+          <t>Grafia brasileira; termo usual na clínica e na genética médica no Brasil; forma de rótulo do HPO (substantivo, só a primeira letra maiúscula, sem ponto final).</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>n_cases / n_genes</t>
+          <t>label_en / definition_en / synonyms_en</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>Em quantos casos e genes do Phenopacket Store o termo aparece. A lista está em ordem decrescente de n_cases.</t>
+          <t>Rótulo, definição e sinônimos oficiais em inglês (HPO). Sinônimos que não são exatos aparecem marcados, por exemplo [related].</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Crédito</t>
+          <t>n_cases / n_genes</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>Nome e ORCID de quem revisar entram como tradutor(a) na submissão ao HPO e como coautor(a) no artigo.</t>
+          <t>Em quantos casos e genes do Phenopacket Store o termo aparece. A lista está em ordem decrescente de n_cases.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Seu nome</t>
-        </is>
-      </c>
-      <c r="B9" s="4" t="inlineStr"/>
+          <t>Crédito</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>Nome e ORCID de quem revisar entram como tradutor(a) na submissão ao HPO e como coautor(a) no artigo.</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
+          <t>Seu nome</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
           <t>Seu ORCID</t>
         </is>
       </c>
-      <c r="B10" s="4" t="inlineStr"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr"/>
+      <c r="B11" s="4" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="inlineStr">
+      <c r="A12" s="2" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
         <is>
           <t>Exemplo de preenchimento (termos que já têm tradução oficial; não fazem parte da lista)</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="5" t="inlineStr">
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
         <is>
           <t>hpo_id</t>
         </is>
       </c>
-      <c r="B13" s="5" t="inlineStr">
+      <c r="B14" s="5" t="inlineStr">
         <is>
           <t>label_en</t>
         </is>
       </c>
-      <c r="C13" s="5" t="inlineStr">
+      <c r="C14" s="5" t="inlineStr">
         <is>
           <t>reviewer_pt</t>
         </is>
       </c>
-      <c r="D13" s="5" t="inlineStr">
+      <c r="D14" s="5" t="inlineStr">
         <is>
           <t>reviewer_notes</t>
         </is>
       </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="6" t="inlineStr">
-        <is>
-          <t>HP:0000252</t>
-        </is>
-      </c>
-      <c r="B14" s="6" t="inlineStr">
-        <is>
-          <t>Microcephaly</t>
-        </is>
-      </c>
-      <c r="C14" s="6" t="inlineStr">
-        <is>
-          <t>Microcefalia</t>
-        </is>
-      </c>
-      <c r="D14" s="6" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="6" t="inlineStr">
         <is>
+          <t>HP:0000252</t>
+        </is>
+      </c>
+      <c r="B15" s="6" t="inlineStr">
+        <is>
+          <t>Microcephaly</t>
+        </is>
+      </c>
+      <c r="C15" s="6" t="inlineStr">
+        <is>
+          <t>Microcefalia</t>
+        </is>
+      </c>
+      <c r="D15" s="6" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="6" t="inlineStr">
+        <is>
           <t>HP:0004322</t>
         </is>
       </c>
-      <c r="B15" s="6" t="inlineStr">
+      <c r="B16" s="6" t="inlineStr">
         <is>
           <t>Short stature</t>
         </is>
       </c>
-      <c r="C15" s="6" t="inlineStr">
+      <c r="C16" s="6" t="inlineStr">
         <is>
           <t>Baixa estatura</t>
         </is>
       </c>
-      <c r="D15" s="6" t="inlineStr"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="2" t="inlineStr">
-        <is>
-          <t>Fontes</t>
-        </is>
-      </c>
-      <c r="B17" s="3" t="inlineStr">
-        <is>
-          <t>HPO v2026-09-01; Phenopacket Store 0.1.27; lista em results/exp02/missing_terms.csv</t>
-        </is>
-      </c>
+      <c r="D16" s="6" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Gerado em</t>
+          <t>Fontes</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25 por reports/build_review.py (commit a12a360)</t>
+          <t>HPO v2026-09-01; Phenopacket Store 0.1.27; lista em results/exp02/missing_terms.csv</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
+          <t>Gerado em</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-25 por reports/build_review.py (commit b2fdad7)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
           <t>Aviso</t>
         </is>
       </c>
-      <c r="B19" s="3" t="inlineStr">
+      <c r="B20" s="3" t="inlineStr">
         <is>
           <t>Apoio à pesquisa; não é ferramenta diagnóstica nem orienta conduta clínica.</t>
         </is>

</xml_diff>

<commit_message>
Add machine-translation candidates for the 50 review terms
Run by the author with claude-opus-5-5 (prompt sha256 2778aaf0b0fc, effort low):
50 API calls, 0 unfinished, US$ 0.3321. Outputs cached in
results/review/translations.jsonl; calls logged in llm_calls.jsonl.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AzLhnR3PoLPQ3QmU5BGcpZ
</commit_message>
<xml_diff>
--- a/reports/review/top50_terms.xlsx
+++ b/reports/review/top50_terms.xlsx
@@ -542,7 +542,7 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>TRADUÇÃO AUTOMÁTICA (gerada por máquina). Exige revisão humana; não usar sem revisão. Fundo laranja. Vazia nesta versão: a variável ANTHROPIC_API_KEY não estava definida. A revisão pode ser feita direto em reviewer_pt.</t>
+          <t>TRADUÇÃO AUTOMÁTICA (gerada por máquina). Exige revisão humana; não usar sem revisão. Fundo laranja. Preenchida para os 50 termos pelo modelo claude-opus-5-5 (prompt prompts/translate_hpo_label_pt_br_v1.system.md, sha256 2778aaf0b0fc).</t>
         </is>
       </c>
     </row>
@@ -698,7 +698,7 @@
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25 por reports/build_review.py (commit b2fdad7)</t>
+          <t>2026-10-25 por reports/build_review.py (commit 6b1ec0b, com mudanças não commitadas)</t>
         </is>
       </c>
     </row>
@@ -813,7 +813,11 @@
       <c r="F2" s="3" t="n">
         <v>254</v>
       </c>
-      <c r="G2" s="8" t="inlineStr"/>
+      <c r="G2" s="8" t="inlineStr">
+        <is>
+          <t>Atraso global do desenvolvimento</t>
+        </is>
+      </c>
       <c r="H2" s="4" t="inlineStr"/>
       <c r="I2" s="4" t="inlineStr"/>
     </row>
@@ -844,7 +848,11 @@
       <c r="F3" s="3" t="n">
         <v>182</v>
       </c>
-      <c r="G3" s="8" t="inlineStr"/>
+      <c r="G3" s="8" t="inlineStr">
+        <is>
+          <t>Atraso no desenvolvimento da fala e da linguagem</t>
+        </is>
+      </c>
       <c r="H3" s="4" t="inlineStr"/>
       <c r="I3" s="4" t="inlineStr"/>
     </row>
@@ -875,7 +883,11 @@
       <c r="F4" s="3" t="n">
         <v>165</v>
       </c>
-      <c r="G4" s="8" t="inlineStr"/>
+      <c r="G4" s="8" t="inlineStr">
+        <is>
+          <t>Deficiência intelectual</t>
+        </is>
+      </c>
       <c r="H4" s="4" t="inlineStr"/>
       <c r="I4" s="4" t="inlineStr"/>
     </row>
@@ -906,7 +918,11 @@
       <c r="F5" s="3" t="n">
         <v>206</v>
       </c>
-      <c r="G5" s="8" t="inlineStr"/>
+      <c r="G5" s="8" t="inlineStr">
+        <is>
+          <t>Hipotonia</t>
+        </is>
+      </c>
       <c r="H5" s="4" t="inlineStr"/>
       <c r="I5" s="4" t="inlineStr"/>
     </row>
@@ -937,7 +953,11 @@
       <c r="F6" s="3" t="n">
         <v>178</v>
       </c>
-      <c r="G6" s="8" t="inlineStr"/>
+      <c r="G6" s="8" t="inlineStr">
+        <is>
+          <t>Crise epiléptica</t>
+        </is>
+      </c>
       <c r="H6" s="4" t="inlineStr"/>
       <c r="I6" s="4" t="inlineStr"/>
     </row>
@@ -968,7 +988,11 @@
       <c r="F7" s="3" t="n">
         <v>121</v>
       </c>
-      <c r="G7" s="8" t="inlineStr"/>
+      <c r="G7" s="8" t="inlineStr">
+        <is>
+          <t>Atraso motor</t>
+        </is>
+      </c>
       <c r="H7" s="4" t="inlineStr"/>
       <c r="I7" s="4" t="inlineStr"/>
     </row>
@@ -999,7 +1023,11 @@
       <c r="F8" s="3" t="n">
         <v>136</v>
       </c>
-      <c r="G8" s="8" t="inlineStr"/>
+      <c r="G8" s="8" t="inlineStr">
+        <is>
+          <t>Dificuldades alimentares</t>
+        </is>
+      </c>
       <c r="H8" s="4" t="inlineStr"/>
       <c r="I8" s="4" t="inlineStr"/>
     </row>
@@ -1030,7 +1058,11 @@
       <c r="F9" s="3" t="n">
         <v>96</v>
       </c>
-      <c r="G9" s="8" t="inlineStr"/>
+      <c r="G9" s="8" t="inlineStr">
+        <is>
+          <t>Atraso na aquisição da marcha</t>
+        </is>
+      </c>
       <c r="H9" s="4" t="inlineStr"/>
       <c r="I9" s="4" t="inlineStr"/>
     </row>
@@ -1061,7 +1093,11 @@
       <c r="F10" s="3" t="n">
         <v>89</v>
       </c>
-      <c r="G10" s="8" t="inlineStr"/>
+      <c r="G10" s="8" t="inlineStr">
+        <is>
+          <t>Comportamento autista</t>
+        </is>
+      </c>
       <c r="H10" s="4" t="inlineStr"/>
       <c r="I10" s="4" t="inlineStr"/>
     </row>
@@ -1092,7 +1128,11 @@
       <c r="F11" s="3" t="n">
         <v>146</v>
       </c>
-      <c r="G11" s="8" t="inlineStr"/>
+      <c r="G11" s="8" t="inlineStr">
+        <is>
+          <t>Escoliose</t>
+        </is>
+      </c>
       <c r="H11" s="4" t="inlineStr"/>
       <c r="I11" s="4" t="inlineStr"/>
     </row>
@@ -1123,7 +1163,11 @@
       <c r="F12" s="3" t="n">
         <v>86</v>
       </c>
-      <c r="G12" s="8" t="inlineStr"/>
+      <c r="G12" s="8" t="inlineStr">
+        <is>
+          <t>Ausência de fala</t>
+        </is>
+      </c>
       <c r="H12" s="4" t="inlineStr"/>
       <c r="I12" s="4" t="inlineStr"/>
     </row>
@@ -1154,7 +1198,11 @@
       <c r="F13" s="3" t="n">
         <v>127</v>
       </c>
-      <c r="G13" s="8" t="inlineStr"/>
+      <c r="G13" s="8" t="inlineStr">
+        <is>
+          <t>Déficit de crescimento</t>
+        </is>
+      </c>
       <c r="H13" s="4" t="inlineStr"/>
       <c r="I13" s="4" t="inlineStr"/>
     </row>
@@ -1185,7 +1233,11 @@
       <c r="F14" s="3" t="n">
         <v>69</v>
       </c>
-      <c r="G14" s="8" t="inlineStr"/>
+      <c r="G14" s="8" t="inlineStr">
+        <is>
+          <t>Deficiência intelectual grave</t>
+        </is>
+      </c>
       <c r="H14" s="4" t="inlineStr"/>
       <c r="I14" s="4" t="inlineStr"/>
     </row>
@@ -1216,7 +1268,11 @@
       <c r="F15" s="3" t="n">
         <v>82</v>
       </c>
-      <c r="G15" s="8" t="inlineStr"/>
+      <c r="G15" s="8" t="inlineStr">
+        <is>
+          <t>Ataxia</t>
+        </is>
+      </c>
       <c r="H15" s="4" t="inlineStr"/>
       <c r="I15" s="4" t="inlineStr"/>
     </row>
@@ -1247,7 +1303,11 @@
       <c r="F16" s="3" t="n">
         <v>78</v>
       </c>
-      <c r="G16" s="8" t="inlineStr"/>
+      <c r="G16" s="8" t="inlineStr">
+        <is>
+          <t>Hipermobilidade articular</t>
+        </is>
+      </c>
       <c r="H16" s="4" t="inlineStr"/>
       <c r="I16" s="4" t="inlineStr"/>
     </row>
@@ -1278,7 +1338,11 @@
       <c r="F17" s="3" t="n">
         <v>101</v>
       </c>
-      <c r="G17" s="8" t="inlineStr"/>
+      <c r="G17" s="8" t="inlineStr">
+        <is>
+          <t>Ponte nasal deprimida</t>
+        </is>
+      </c>
       <c r="H17" s="4" t="inlineStr"/>
       <c r="I17" s="4" t="inlineStr"/>
     </row>
@@ -1309,7 +1373,11 @@
       <c r="F18" s="3" t="n">
         <v>99</v>
       </c>
-      <c r="G18" s="8" t="inlineStr"/>
+      <c r="G18" s="8" t="inlineStr">
+        <is>
+          <t>Corpo caloso fino</t>
+        </is>
+      </c>
       <c r="H18" s="4" t="inlineStr"/>
       <c r="I18" s="4" t="inlineStr"/>
     </row>
@@ -1340,7 +1408,11 @@
       <c r="F19" s="3" t="n">
         <v>72</v>
       </c>
-      <c r="G19" s="8" t="inlineStr"/>
+      <c r="G19" s="8" t="inlineStr">
+        <is>
+          <t>Pé plano</t>
+        </is>
+      </c>
       <c r="H19" s="4" t="inlineStr"/>
       <c r="I19" s="4" t="inlineStr"/>
     </row>
@@ -1371,7 +1443,11 @@
       <c r="F20" s="3" t="n">
         <v>65</v>
       </c>
-      <c r="G20" s="8" t="inlineStr"/>
+      <c r="G20" s="8" t="inlineStr">
+        <is>
+          <t>Atrofia cerebelar</t>
+        </is>
+      </c>
       <c r="H20" s="4" t="inlineStr"/>
       <c r="I20" s="4" t="inlineStr"/>
     </row>
@@ -1402,7 +1478,11 @@
       <c r="F21" s="3" t="n">
         <v>82</v>
       </c>
-      <c r="G21" s="8" t="inlineStr"/>
+      <c r="G21" s="8" t="inlineStr">
+        <is>
+          <t>Deficiência auditiva</t>
+        </is>
+      </c>
       <c r="H21" s="4" t="inlineStr"/>
       <c r="I21" s="4" t="inlineStr"/>
     </row>
@@ -1433,7 +1513,11 @@
       <c r="F22" s="3" t="n">
         <v>80</v>
       </c>
-      <c r="G22" s="8" t="inlineStr"/>
+      <c r="G22" s="8" t="inlineStr">
+        <is>
+          <t>Deficiência intelectual leve</t>
+        </is>
+      </c>
       <c r="H22" s="4" t="inlineStr"/>
       <c r="I22" s="4" t="inlineStr"/>
     </row>
@@ -1464,7 +1548,11 @@
       <c r="F23" s="3" t="n">
         <v>58</v>
       </c>
-      <c r="G23" s="8" t="inlineStr"/>
+      <c r="G23" s="8" t="inlineStr">
+        <is>
+          <t>Disartria</t>
+        </is>
+      </c>
       <c r="H23" s="4" t="inlineStr"/>
       <c r="I23" s="4" t="inlineStr"/>
     </row>
@@ -1495,7 +1583,11 @@
       <c r="F24" s="3" t="n">
         <v>55</v>
       </c>
-      <c r="G24" s="8" t="inlineStr"/>
+      <c r="G24" s="8" t="inlineStr">
+        <is>
+          <t>Crise tônico-clônica bilateral</t>
+        </is>
+      </c>
       <c r="H24" s="4" t="inlineStr"/>
       <c r="I24" s="4" t="inlineStr"/>
     </row>
@@ -1526,7 +1618,11 @@
       <c r="F25" s="3" t="n">
         <v>44</v>
       </c>
-      <c r="G25" s="8" t="inlineStr"/>
+      <c r="G25" s="8" t="inlineStr">
+        <is>
+          <t>Atraso global do desenvolvimento grave</t>
+        </is>
+      </c>
       <c r="H25" s="4" t="inlineStr"/>
       <c r="I25" s="4" t="inlineStr"/>
     </row>
@@ -1557,7 +1653,11 @@
       <c r="F26" s="3" t="n">
         <v>77</v>
       </c>
-      <c r="G26" s="8" t="inlineStr"/>
+      <c r="G26" s="8" t="inlineStr">
+        <is>
+          <t>Comunicação interatrial</t>
+        </is>
+      </c>
       <c r="H26" s="4" t="inlineStr"/>
       <c r="I26" s="4" t="inlineStr"/>
     </row>
@@ -1588,7 +1688,11 @@
       <c r="F27" s="3" t="n">
         <v>80</v>
       </c>
-      <c r="G27" s="8" t="inlineStr"/>
+      <c r="G27" s="8" t="inlineStr">
+        <is>
+          <t>Restrição de crescimento intrauterino</t>
+        </is>
+      </c>
       <c r="H27" s="4" t="inlineStr"/>
       <c r="I27" s="4" t="inlineStr"/>
     </row>
@@ -1619,7 +1723,11 @@
       <c r="F28" s="3" t="n">
         <v>64</v>
       </c>
-      <c r="G28" s="8" t="inlineStr"/>
+      <c r="G28" s="8" t="inlineStr">
+        <is>
+          <t>Deficiência intelectual moderada</t>
+        </is>
+      </c>
       <c r="H28" s="4" t="inlineStr"/>
       <c r="I28" s="4" t="inlineStr"/>
     </row>
@@ -1650,7 +1758,11 @@
       <c r="F29" s="3" t="n">
         <v>36</v>
       </c>
-      <c r="G29" s="8" t="inlineStr"/>
+      <c r="G29" s="8" t="inlineStr">
+        <is>
+          <t>Atraso do desenvolvimento motor grosso</t>
+        </is>
+      </c>
       <c r="H29" s="4" t="inlineStr"/>
       <c r="I29" s="4" t="inlineStr"/>
     </row>
@@ -1681,7 +1793,11 @@
       <c r="F30" s="3" t="n">
         <v>55</v>
       </c>
-      <c r="G30" s="8" t="inlineStr"/>
+      <c r="G30" s="8" t="inlineStr">
+        <is>
+          <t>Regressão do desenvolvimento</t>
+        </is>
+      </c>
       <c r="H30" s="4" t="inlineStr"/>
       <c r="I30" s="4" t="inlineStr"/>
     </row>
@@ -1712,7 +1828,11 @@
       <c r="F31" s="3" t="n">
         <v>63</v>
       </c>
-      <c r="G31" s="8" t="inlineStr"/>
+      <c r="G31" s="8" t="inlineStr">
+        <is>
+          <t>Hipotonia axial</t>
+        </is>
+      </c>
       <c r="H31" s="4" t="inlineStr"/>
       <c r="I31" s="4" t="inlineStr"/>
     </row>
@@ -1743,7 +1863,11 @@
       <c r="F32" s="3" t="n">
         <v>66</v>
       </c>
-      <c r="G32" s="8" t="inlineStr"/>
+      <c r="G32" s="8" t="inlineStr">
+        <is>
+          <t>Refluxo gastroesofágico</t>
+        </is>
+      </c>
       <c r="H32" s="4" t="inlineStr"/>
       <c r="I32" s="4" t="inlineStr"/>
     </row>
@@ -1774,7 +1898,11 @@
       <c r="F33" s="3" t="n">
         <v>73</v>
       </c>
-      <c r="G33" s="8" t="inlineStr"/>
+      <c r="G33" s="8" t="inlineStr">
+        <is>
+          <t>Ventriculomegalia</t>
+        </is>
+      </c>
       <c r="H33" s="4" t="inlineStr"/>
       <c r="I33" s="4" t="inlineStr"/>
     </row>
@@ -1805,7 +1933,11 @@
       <c r="F34" s="3" t="n">
         <v>83</v>
       </c>
-      <c r="G34" s="8" t="inlineStr"/>
+      <c r="G34" s="8" t="inlineStr">
+        <is>
+          <t>Comunicação interventricular</t>
+        </is>
+      </c>
       <c r="H34" s="4" t="inlineStr"/>
       <c r="I34" s="4" t="inlineStr"/>
     </row>
@@ -1836,7 +1968,11 @@
       <c r="F35" s="3" t="n">
         <v>42</v>
       </c>
-      <c r="G35" s="8" t="inlineStr"/>
+      <c r="G35" s="8" t="inlineStr">
+        <is>
+          <t>Sobrancelha muito arqueada</t>
+        </is>
+      </c>
       <c r="H35" s="4" t="inlineStr"/>
       <c r="I35" s="4" t="inlineStr"/>
     </row>
@@ -1867,7 +2003,11 @@
       <c r="F36" s="3" t="n">
         <v>66</v>
       </c>
-      <c r="G36" s="8" t="inlineStr"/>
+      <c r="G36" s="8" t="inlineStr">
+        <is>
+          <t>Espasticidade</t>
+        </is>
+      </c>
       <c r="H36" s="4" t="inlineStr"/>
       <c r="I36" s="4" t="inlineStr"/>
     </row>
@@ -1898,7 +2038,11 @@
       <c r="F37" s="3" t="n">
         <v>67</v>
       </c>
-      <c r="G37" s="8" t="inlineStr"/>
+      <c r="G37" s="8" t="inlineStr">
+        <is>
+          <t>Pectus excavatum</t>
+        </is>
+      </c>
       <c r="H37" s="4" t="inlineStr"/>
       <c r="I37" s="4" t="inlineStr"/>
     </row>
@@ -1929,7 +2073,11 @@
       <c r="F38" s="3" t="n">
         <v>52</v>
       </c>
-      <c r="G38" s="8" t="inlineStr"/>
+      <c r="G38" s="8" t="inlineStr">
+        <is>
+          <t>Sinofris</t>
+        </is>
+      </c>
       <c r="H38" s="4" t="inlineStr"/>
       <c r="I38" s="4" t="inlineStr"/>
     </row>
@@ -1960,7 +2108,11 @@
       <c r="F39" s="3" t="n">
         <v>8</v>
       </c>
-      <c r="G39" s="8" t="inlineStr"/>
+      <c r="G39" s="8" t="inlineStr">
+        <is>
+          <t>Macrodontia</t>
+        </is>
+      </c>
       <c r="H39" s="4" t="inlineStr"/>
       <c r="I39" s="4" t="inlineStr"/>
     </row>
@@ -1991,7 +2143,11 @@
       <c r="F40" s="3" t="n">
         <v>31</v>
       </c>
-      <c r="G40" s="8" t="inlineStr"/>
+      <c r="G40" s="8" t="inlineStr">
+        <is>
+          <t>Anormalidade no EEG</t>
+        </is>
+      </c>
       <c r="H40" s="4" t="inlineStr"/>
       <c r="I40" s="4" t="inlineStr"/>
     </row>
@@ -2022,7 +2178,11 @@
       <c r="F41" s="3" t="n">
         <v>46</v>
       </c>
-      <c r="G41" s="8" t="inlineStr"/>
+      <c r="G41" s="8" t="inlineStr">
+        <is>
+          <t>Fronte proeminente</t>
+        </is>
+      </c>
       <c r="H41" s="4" t="inlineStr"/>
       <c r="I41" s="4" t="inlineStr"/>
     </row>
@@ -2049,7 +2209,11 @@
       <c r="F42" s="3" t="n">
         <v>47</v>
       </c>
-      <c r="G42" s="8" t="inlineStr"/>
+      <c r="G42" s="8" t="inlineStr">
+        <is>
+          <t>Atraso na aquisição do sentar</t>
+        </is>
+      </c>
       <c r="H42" s="4" t="inlineStr"/>
       <c r="I42" s="4" t="inlineStr"/>
     </row>
@@ -2080,7 +2244,11 @@
       <c r="F43" s="3" t="n">
         <v>55</v>
       </c>
-      <c r="G43" s="8" t="inlineStr"/>
+      <c r="G43" s="8" t="inlineStr">
+        <is>
+          <t>Hiper-reflexia</t>
+        </is>
+      </c>
       <c r="H43" s="4" t="inlineStr"/>
       <c r="I43" s="4" t="inlineStr"/>
     </row>
@@ -2107,7 +2275,11 @@
       <c r="F44" s="3" t="n">
         <v>41</v>
       </c>
-      <c r="G44" s="8" t="inlineStr"/>
+      <c r="G44" s="8" t="inlineStr">
+        <is>
+          <t>Autismo</t>
+        </is>
+      </c>
       <c r="H44" s="4" t="inlineStr"/>
       <c r="I44" s="4" t="inlineStr"/>
     </row>
@@ -2138,7 +2310,11 @@
       <c r="F45" s="3" t="n">
         <v>63</v>
       </c>
-      <c r="G45" s="8" t="inlineStr"/>
+      <c r="G45" s="8" t="inlineStr">
+        <is>
+          <t>Comportamento agressivo</t>
+        </is>
+      </c>
       <c r="H45" s="4" t="inlineStr"/>
       <c r="I45" s="4" t="inlineStr"/>
     </row>
@@ -2169,7 +2345,11 @@
       <c r="F46" s="3" t="n">
         <v>50</v>
       </c>
-      <c r="G46" s="8" t="inlineStr"/>
+      <c r="G46" s="8" t="inlineStr">
+        <is>
+          <t>Retrusão do terço médio da face</t>
+        </is>
+      </c>
       <c r="H46" s="4" t="inlineStr"/>
       <c r="I46" s="4" t="inlineStr"/>
     </row>
@@ -2200,7 +2380,11 @@
       <c r="F47" s="3" t="n">
         <v>47</v>
       </c>
-      <c r="G47" s="8" t="inlineStr"/>
+      <c r="G47" s="8" t="inlineStr">
+        <is>
+          <t>Distúrbio da marcha</t>
+        </is>
+      </c>
       <c r="H47" s="4" t="inlineStr"/>
       <c r="I47" s="4" t="inlineStr"/>
     </row>
@@ -2231,7 +2415,11 @@
       <c r="F48" s="3" t="n">
         <v>52</v>
       </c>
-      <c r="G48" s="8" t="inlineStr"/>
+      <c r="G48" s="8" t="inlineStr">
+        <is>
+          <t>Braquidactilia</t>
+        </is>
+      </c>
       <c r="H48" s="4" t="inlineStr"/>
       <c r="I48" s="4" t="inlineStr"/>
     </row>
@@ -2262,7 +2450,11 @@
       <c r="F49" s="3" t="n">
         <v>56</v>
       </c>
-      <c r="G49" s="8" t="inlineStr"/>
+      <c r="G49" s="8" t="inlineStr">
+        <is>
+          <t>Atrofia cerebral</t>
+        </is>
+      </c>
       <c r="H49" s="4" t="inlineStr"/>
       <c r="I49" s="4" t="inlineStr"/>
     </row>
@@ -2293,7 +2485,11 @@
       <c r="F50" s="3" t="n">
         <v>20</v>
       </c>
-      <c r="G50" s="8" t="inlineStr"/>
+      <c r="G50" s="8" t="inlineStr">
+        <is>
+          <t>Concentração circulante de lactato aumentada</t>
+        </is>
+      </c>
       <c r="H50" s="4" t="inlineStr"/>
       <c r="I50" s="4" t="inlineStr"/>
     </row>
@@ -2324,7 +2520,11 @@
       <c r="F51" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="G51" s="8" t="inlineStr"/>
+      <c r="G51" s="8" t="inlineStr">
+        <is>
+          <t>Anormalidade da mão</t>
+        </is>
+      </c>
       <c r="H51" s="4" t="inlineStr"/>
       <c r="I51" s="4" t="inlineStr"/>
     </row>

</xml_diff>

<commit_message>
Regenerate review package with author notes
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AzLhnR3PoLPQ3QmU5BGcpZ
</commit_message>
<xml_diff>
--- a/reports/review/top50_terms.xlsx
+++ b/reports/review/top50_terms.xlsx
@@ -11,7 +11,7 @@
     <sheet name="termos" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'termos'!$A$1:$I$51</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'termos'!$A$1:$J$51</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -48,7 +48,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -70,6 +70,11 @@
         <fgColor rgb="00FCE4D6"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DDEBF7"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -83,7 +88,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -99,6 +104,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -190,10 +198,15 @@
     </comment>
     <comment ref="H1" authorId="0" shapeId="0">
       <text>
+        <t>Observações do autor do projeto: sugestões, não decisões.</t>
+      </text>
+    </comment>
+    <comment ref="I1" authorId="0" shapeId="0">
+      <text>
         <t>Preencha com o rótulo final em PT-BR (mesmo que igual ao candidato).</t>
       </text>
     </comment>
-    <comment ref="I1" authorId="0" shapeId="0">
+    <comment ref="J1" authorId="0" shapeId="0">
       <text>
         <t>Opcional: dúvidas, termo alternativo, uso regional. Se mantiver a candidata sem mudar nada, escreva: candidata aceita sem alteração</t>
       </text>
@@ -491,7 +504,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D20"/>
+  <dimension ref="A1:D21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -549,166 +562,178 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Convenções</t>
+          <t>author_notes</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>Grafia brasileira; termo usual na clínica e na genética médica no Brasil; forma de rótulo do HPO (substantivo, só a primeira letra maiúscula, sem ponto final).</t>
+          <t>Observações do autor do projeto em 6 termos: padronização com a tradução oficial do HPO e escolhas clínicas em aberto. Fundo azul. São sugestões, não decisões; o rótulo final é seu.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>label_en / definition_en / synonyms_en</t>
+          <t>Convenções</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>Rótulo, definição e sinônimos oficiais em inglês (HPO). Sinônimos que não são exatos aparecem marcados, por exemplo [related].</t>
+          <t>Grafia brasileira; termo usual na clínica e na genética médica no Brasil; forma de rótulo do HPO (substantivo, só a primeira letra maiúscula, sem ponto final).</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>n_cases / n_genes</t>
+          <t>label_en / definition_en / synonyms_en</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>Em quantos casos e genes do Phenopacket Store o termo aparece. A lista está em ordem decrescente de n_cases.</t>
+          <t>Rótulo, definição e sinônimos oficiais em inglês (HPO). Sinônimos que não são exatos aparecem marcados, por exemplo [related].</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Crédito</t>
+          <t>n_cases / n_genes</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>Nome e ORCID de quem revisar entram como tradutor(a) na submissão ao HPO e como coautor(a) no artigo.</t>
+          <t>Em quantos casos e genes do Phenopacket Store o termo aparece. A lista está em ordem decrescente de n_cases.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Seu nome</t>
-        </is>
-      </c>
-      <c r="B10" s="4" t="inlineStr"/>
+          <t>Crédito</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>Nome e ORCID de quem revisar entram como tradutor(a) na submissão ao HPO e como coautor(a) no artigo.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
+          <t>Seu nome</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
           <t>Seu ORCID</t>
         </is>
       </c>
-      <c r="B11" s="4" t="inlineStr"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr"/>
+      <c r="B12" s="4" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" s="2" t="inlineStr">
+      <c r="A13" s="2" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
         <is>
           <t>Exemplo de preenchimento (termos que já têm tradução oficial; não fazem parte da lista)</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="5" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
         <is>
           <t>hpo_id</t>
         </is>
       </c>
-      <c r="B14" s="5" t="inlineStr">
+      <c r="B15" s="5" t="inlineStr">
         <is>
           <t>label_en</t>
         </is>
       </c>
-      <c r="C14" s="5" t="inlineStr">
+      <c r="C15" s="5" t="inlineStr">
         <is>
           <t>reviewer_pt</t>
         </is>
       </c>
-      <c r="D14" s="5" t="inlineStr">
+      <c r="D15" s="5" t="inlineStr">
         <is>
           <t>reviewer_notes</t>
         </is>
       </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="6" t="inlineStr">
-        <is>
-          <t>HP:0000252</t>
-        </is>
-      </c>
-      <c r="B15" s="6" t="inlineStr">
-        <is>
-          <t>Microcephaly</t>
-        </is>
-      </c>
-      <c r="C15" s="6" t="inlineStr">
-        <is>
-          <t>Microcefalia</t>
-        </is>
-      </c>
-      <c r="D15" s="6" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
         <is>
+          <t>HP:0000252</t>
+        </is>
+      </c>
+      <c r="B16" s="6" t="inlineStr">
+        <is>
+          <t>Microcephaly</t>
+        </is>
+      </c>
+      <c r="C16" s="6" t="inlineStr">
+        <is>
+          <t>Microcefalia</t>
+        </is>
+      </c>
+      <c r="D16" s="6" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="6" t="inlineStr">
+        <is>
           <t>HP:0004322</t>
         </is>
       </c>
-      <c r="B16" s="6" t="inlineStr">
+      <c r="B17" s="6" t="inlineStr">
         <is>
           <t>Short stature</t>
         </is>
       </c>
-      <c r="C16" s="6" t="inlineStr">
+      <c r="C17" s="6" t="inlineStr">
         <is>
           <t>Baixa estatura</t>
         </is>
       </c>
-      <c r="D16" s="6" t="inlineStr"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="2" t="inlineStr">
-        <is>
-          <t>Fontes</t>
-        </is>
-      </c>
-      <c r="B18" s="3" t="inlineStr">
-        <is>
-          <t>HPO v2026-09-01; Phenopacket Store 0.1.27; lista em results/exp02/missing_terms.csv</t>
-        </is>
-      </c>
+      <c r="D17" s="6" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Gerado em</t>
+          <t>Fontes</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>2026-10-25 por reports/build_review.py (commit 79a1f34)</t>
+          <t>HPO v2026-09-01; Phenopacket Store 0.1.27; lista em results/exp02/missing_terms.csv</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
+          <t>Gerado em</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-26 por reports/build_review.py (commit 045d94e)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
           <t>Aviso</t>
         </is>
       </c>
-      <c r="B20" s="3" t="inlineStr">
+      <c r="B21" s="3" t="inlineStr">
         <is>
           <t>Apoio à pesquisa; não é ferramenta diagnóstica nem orienta conduta clínica.</t>
         </is>
@@ -725,7 +750,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I51"/>
+  <dimension ref="A1:J51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -735,8 +760,9 @@
     <col width="9" customWidth="1" min="5" max="5"/>
     <col width="9" customWidth="1" min="6" max="6"/>
     <col width="32" customWidth="1" min="7" max="7"/>
-    <col width="32" customWidth="1" min="8" max="8"/>
-    <col width="40" customWidth="1" min="9" max="9"/>
+    <col width="50" customWidth="1" min="8" max="8"/>
+    <col width="32" customWidth="1" min="9" max="9"/>
+    <col width="40" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -777,10 +803,15 @@
       </c>
       <c r="H1" s="7" t="inlineStr">
         <is>
+          <t>author_notes</t>
+        </is>
+      </c>
+      <c r="I1" s="7" t="inlineStr">
+        <is>
           <t>reviewer_pt</t>
         </is>
       </c>
-      <c r="I1" s="7" t="inlineStr">
+      <c r="J1" s="7" t="inlineStr">
         <is>
           <t>reviewer_notes</t>
         </is>
@@ -818,8 +849,9 @@
           <t>Atraso global do desenvolvimento</t>
         </is>
       </c>
-      <c r="H2" s="4" t="inlineStr"/>
+      <c r="H2" s="9" t="inlineStr"/>
       <c r="I2" s="4" t="inlineStr"/>
+      <c r="J2" s="4" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
@@ -853,8 +885,9 @@
           <t>Atraso no desenvolvimento da fala e da linguagem</t>
         </is>
       </c>
-      <c r="H3" s="4" t="inlineStr"/>
+      <c r="H3" s="9" t="inlineStr"/>
       <c r="I3" s="4" t="inlineStr"/>
+      <c r="J3" s="4" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
@@ -888,8 +921,9 @@
           <t>Deficiência intelectual</t>
         </is>
       </c>
-      <c r="H4" s="4" t="inlineStr"/>
+      <c r="H4" s="9" t="inlineStr"/>
       <c r="I4" s="4" t="inlineStr"/>
+      <c r="J4" s="4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -923,8 +957,9 @@
           <t>Hipotonia</t>
         </is>
       </c>
-      <c r="H5" s="4" t="inlineStr"/>
+      <c r="H5" s="9" t="inlineStr"/>
       <c r="I5" s="4" t="inlineStr"/>
+      <c r="J5" s="4" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
@@ -958,8 +993,13 @@
           <t>Crise epiléptica</t>
         </is>
       </c>
-      <c r="H6" s="4" t="inlineStr"/>
+      <c r="H6" s="9" t="inlineStr">
+        <is>
+          <t>Decisão clínica: 'Crise epiléptica' ou outro termo? No HPO, 'Epileptic seizure' é sinônimo exato, e o termo inclui crises não motoras (ex.: HP:0002121, ausência); 'Crise convulsiva' pode estreitar o conceito. Nos rótulos oficiais deste ramo, 233 de 284 começam com 'Crise epiléptica' e 11 com 'Convulsão'.</t>
+        </is>
+      </c>
       <c r="I6" s="4" t="inlineStr"/>
+      <c r="J6" s="4" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
@@ -993,8 +1033,9 @@
           <t>Atraso motor</t>
         </is>
       </c>
-      <c r="H7" s="4" t="inlineStr"/>
+      <c r="H7" s="9" t="inlineStr"/>
       <c r="I7" s="4" t="inlineStr"/>
+      <c r="J7" s="4" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
@@ -1028,8 +1069,9 @@
           <t>Dificuldades alimentares</t>
         </is>
       </c>
-      <c r="H8" s="4" t="inlineStr"/>
+      <c r="H8" s="9" t="inlineStr"/>
       <c r="I8" s="4" t="inlineStr"/>
+      <c r="J8" s="4" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
@@ -1063,8 +1105,9 @@
           <t>Atraso na aquisição da marcha</t>
         </is>
       </c>
-      <c r="H9" s="4" t="inlineStr"/>
+      <c r="H9" s="9" t="inlineStr"/>
       <c r="I9" s="4" t="inlineStr"/>
+      <c r="J9" s="4" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
@@ -1098,8 +1141,9 @@
           <t>Comportamento autista</t>
         </is>
       </c>
-      <c r="H10" s="4" t="inlineStr"/>
+      <c r="H10" s="9" t="inlineStr"/>
       <c r="I10" s="4" t="inlineStr"/>
+      <c r="J10" s="4" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
@@ -1133,8 +1177,9 @@
           <t>Escoliose</t>
         </is>
       </c>
-      <c r="H11" s="4" t="inlineStr"/>
+      <c r="H11" s="9" t="inlineStr"/>
       <c r="I11" s="4" t="inlineStr"/>
+      <c r="J11" s="4" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
@@ -1168,8 +1213,9 @@
           <t>Ausência de fala</t>
         </is>
       </c>
-      <c r="H12" s="4" t="inlineStr"/>
+      <c r="H12" s="9" t="inlineStr"/>
       <c r="I12" s="4" t="inlineStr"/>
+      <c r="J12" s="4" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
@@ -1203,8 +1249,13 @@
           <t>Déficit de crescimento</t>
         </is>
       </c>
-      <c r="H13" s="4" t="inlineStr"/>
+      <c r="H13" s="9" t="inlineStr">
+        <is>
+          <t>Pedimos sua opinião: no Brasil também se usa 'baixo ganho ponderal'. No HPO, 'Poor weight gain' é só sinônimo relacionado [related]; os exatos incluem 'Weight faltering' e 'Postnatal failure to thrive'. A escolha vale também para termos ainda sem tradução: HP:0001525 (Severe failure to thrive), HP:0001531 (Failure to thrive in infancy), HP:0008866 (Failure to thrive secondary to recurrent infections).</t>
+        </is>
+      </c>
       <c r="I13" s="4" t="inlineStr"/>
+      <c r="J13" s="4" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
@@ -1238,8 +1289,9 @@
           <t>Deficiência intelectual grave</t>
         </is>
       </c>
-      <c r="H14" s="4" t="inlineStr"/>
+      <c r="H14" s="9" t="inlineStr"/>
       <c r="I14" s="4" t="inlineStr"/>
+      <c r="J14" s="4" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
@@ -1273,8 +1325,9 @@
           <t>Ataxia</t>
         </is>
       </c>
-      <c r="H15" s="4" t="inlineStr"/>
+      <c r="H15" s="9" t="inlineStr"/>
       <c r="I15" s="4" t="inlineStr"/>
+      <c r="J15" s="4" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
@@ -1308,8 +1361,9 @@
           <t>Hipermobilidade articular</t>
         </is>
       </c>
-      <c r="H16" s="4" t="inlineStr"/>
+      <c r="H16" s="9" t="inlineStr"/>
       <c r="I16" s="4" t="inlineStr"/>
+      <c r="J16" s="4" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
@@ -1343,8 +1397,9 @@
           <t>Ponte nasal deprimida</t>
         </is>
       </c>
-      <c r="H17" s="4" t="inlineStr"/>
+      <c r="H17" s="9" t="inlineStr"/>
       <c r="I17" s="4" t="inlineStr"/>
+      <c r="J17" s="4" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
@@ -1378,8 +1433,9 @@
           <t>Corpo caloso fino</t>
         </is>
       </c>
-      <c r="H18" s="4" t="inlineStr"/>
+      <c r="H18" s="9" t="inlineStr"/>
       <c r="I18" s="4" t="inlineStr"/>
+      <c r="J18" s="4" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
@@ -1413,8 +1469,9 @@
           <t>Pé plano</t>
         </is>
       </c>
-      <c r="H19" s="4" t="inlineStr"/>
+      <c r="H19" s="9" t="inlineStr"/>
       <c r="I19" s="4" t="inlineStr"/>
+      <c r="J19" s="4" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
@@ -1448,8 +1505,9 @@
           <t>Atrofia cerebelar</t>
         </is>
       </c>
-      <c r="H20" s="4" t="inlineStr"/>
+      <c r="H20" s="9" t="inlineStr"/>
       <c r="I20" s="4" t="inlineStr"/>
+      <c r="J20" s="4" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
@@ -1483,8 +1541,9 @@
           <t>Deficiência auditiva</t>
         </is>
       </c>
-      <c r="H21" s="4" t="inlineStr"/>
+      <c r="H21" s="9" t="inlineStr"/>
       <c r="I21" s="4" t="inlineStr"/>
+      <c r="J21" s="4" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
@@ -1518,8 +1577,9 @@
           <t>Deficiência intelectual leve</t>
         </is>
       </c>
-      <c r="H22" s="4" t="inlineStr"/>
+      <c r="H22" s="9" t="inlineStr"/>
       <c r="I22" s="4" t="inlineStr"/>
+      <c r="J22" s="4" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
@@ -1553,8 +1613,9 @@
           <t>Disartria</t>
         </is>
       </c>
-      <c r="H23" s="4" t="inlineStr"/>
+      <c r="H23" s="9" t="inlineStr"/>
       <c r="I23" s="4" t="inlineStr"/>
+      <c r="J23" s="4" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
@@ -1588,8 +1649,13 @@
           <t>Crise tônico-clônica bilateral</t>
         </is>
       </c>
-      <c r="H24" s="4" t="inlineStr"/>
+      <c r="H24" s="9" t="inlineStr">
+        <is>
+          <t>Consistência: 3 dos 6 termos abaixo dele no HPO que já têm tradução usam 'Convulsão tônico-clônica ...' (ex.: HP:0007193, 'Convulsão tônico-clônica bilateral ao despertar'). Vale alinhar 'Crise' ou 'Convulsão' com a escolha para HP:0001250 (Seizure).</t>
+        </is>
+      </c>
       <c r="I24" s="4" t="inlineStr"/>
+      <c r="J24" s="4" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
@@ -1623,8 +1689,9 @@
           <t>Atraso global do desenvolvimento grave</t>
         </is>
       </c>
-      <c r="H25" s="4" t="inlineStr"/>
+      <c r="H25" s="9" t="inlineStr"/>
       <c r="I25" s="4" t="inlineStr"/>
+      <c r="J25" s="4" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
@@ -1658,8 +1725,9 @@
           <t>Comunicação interatrial</t>
         </is>
       </c>
-      <c r="H26" s="4" t="inlineStr"/>
+      <c r="H26" s="9" t="inlineStr"/>
       <c r="I26" s="4" t="inlineStr"/>
+      <c r="J26" s="4" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
@@ -1693,8 +1761,9 @@
           <t>Restrição de crescimento intrauterino</t>
         </is>
       </c>
-      <c r="H27" s="4" t="inlineStr"/>
+      <c r="H27" s="9" t="inlineStr"/>
       <c r="I27" s="4" t="inlineStr"/>
+      <c r="J27" s="4" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
@@ -1728,8 +1797,9 @@
           <t>Deficiência intelectual moderada</t>
         </is>
       </c>
-      <c r="H28" s="4" t="inlineStr"/>
+      <c r="H28" s="9" t="inlineStr"/>
       <c r="I28" s="4" t="inlineStr"/>
+      <c r="J28" s="4" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
@@ -1763,8 +1833,9 @@
           <t>Atraso do desenvolvimento motor grosso</t>
         </is>
       </c>
-      <c r="H29" s="4" t="inlineStr"/>
+      <c r="H29" s="9" t="inlineStr"/>
       <c r="I29" s="4" t="inlineStr"/>
+      <c r="J29" s="4" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="3" t="inlineStr">
@@ -1798,8 +1869,9 @@
           <t>Regressão do desenvolvimento</t>
         </is>
       </c>
-      <c r="H30" s="4" t="inlineStr"/>
+      <c r="H30" s="9" t="inlineStr"/>
       <c r="I30" s="4" t="inlineStr"/>
+      <c r="J30" s="4" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
@@ -1833,8 +1905,9 @@
           <t>Hipotonia axial</t>
         </is>
       </c>
-      <c r="H31" s="4" t="inlineStr"/>
+      <c r="H31" s="9" t="inlineStr"/>
       <c r="I31" s="4" t="inlineStr"/>
+      <c r="J31" s="4" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="3" t="inlineStr">
@@ -1868,8 +1941,9 @@
           <t>Refluxo gastroesofágico</t>
         </is>
       </c>
-      <c r="H32" s="4" t="inlineStr"/>
+      <c r="H32" s="9" t="inlineStr"/>
       <c r="I32" s="4" t="inlineStr"/>
+      <c r="J32" s="4" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
@@ -1903,8 +1977,9 @@
           <t>Ventriculomegalia</t>
         </is>
       </c>
-      <c r="H33" s="4" t="inlineStr"/>
+      <c r="H33" s="9" t="inlineStr"/>
       <c r="I33" s="4" t="inlineStr"/>
+      <c r="J33" s="4" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="3" t="inlineStr">
@@ -1938,8 +2013,9 @@
           <t>Comunicação interventricular</t>
         </is>
       </c>
-      <c r="H34" s="4" t="inlineStr"/>
+      <c r="H34" s="9" t="inlineStr"/>
       <c r="I34" s="4" t="inlineStr"/>
+      <c r="J34" s="4" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
@@ -1973,8 +2049,9 @@
           <t>Sobrancelha muito arqueada</t>
         </is>
       </c>
-      <c r="H35" s="4" t="inlineStr"/>
+      <c r="H35" s="9" t="inlineStr"/>
       <c r="I35" s="4" t="inlineStr"/>
+      <c r="J35" s="4" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="3" t="inlineStr">
@@ -2008,8 +2085,9 @@
           <t>Espasticidade</t>
         </is>
       </c>
-      <c r="H36" s="4" t="inlineStr"/>
+      <c r="H36" s="9" t="inlineStr"/>
       <c r="I36" s="4" t="inlineStr"/>
+      <c r="J36" s="4" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="3" t="inlineStr">
@@ -2043,8 +2121,9 @@
           <t>Pectus excavatum</t>
         </is>
       </c>
-      <c r="H37" s="4" t="inlineStr"/>
+      <c r="H37" s="9" t="inlineStr"/>
       <c r="I37" s="4" t="inlineStr"/>
+      <c r="J37" s="4" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="3" t="inlineStr">
@@ -2078,8 +2157,9 @@
           <t>Sinofris</t>
         </is>
       </c>
-      <c r="H38" s="4" t="inlineStr"/>
+      <c r="H38" s="9" t="inlineStr"/>
       <c r="I38" s="4" t="inlineStr"/>
+      <c r="J38" s="4" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="3" t="inlineStr">
@@ -2113,8 +2193,9 @@
           <t>Macrodontia</t>
         </is>
       </c>
-      <c r="H39" s="4" t="inlineStr"/>
+      <c r="H39" s="9" t="inlineStr"/>
       <c r="I39" s="4" t="inlineStr"/>
+      <c r="J39" s="4" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="3" t="inlineStr">
@@ -2148,8 +2229,13 @@
           <t>Anormalidade no EEG</t>
         </is>
       </c>
-      <c r="H40" s="4" t="inlineStr"/>
+      <c r="H40" s="9" t="inlineStr">
+        <is>
+          <t>Padronização: a tradução oficial do HPO usa 'Anomalia', não 'Anormalidade'. 264 rótulos oficiais começam com 'Anomalia' e 0 com 'Anormalidade'; dos 201 termos 'Abnormality of ...' já traduzidos, 200 começam com 'Anomalia' (ex.: HP:0000002, 'Anomalia da altura corporal').</t>
+        </is>
+      </c>
       <c r="I40" s="4" t="inlineStr"/>
+      <c r="J40" s="4" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="3" t="inlineStr">
@@ -2183,8 +2269,9 @@
           <t>Fronte proeminente</t>
         </is>
       </c>
-      <c r="H41" s="4" t="inlineStr"/>
+      <c r="H41" s="9" t="inlineStr"/>
       <c r="I41" s="4" t="inlineStr"/>
+      <c r="J41" s="4" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="3" t="inlineStr">
@@ -2214,8 +2301,9 @@
           <t>Atraso na aquisição do sentar</t>
         </is>
       </c>
-      <c r="H42" s="4" t="inlineStr"/>
+      <c r="H42" s="9" t="inlineStr"/>
       <c r="I42" s="4" t="inlineStr"/>
+      <c r="J42" s="4" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" s="3" t="inlineStr">
@@ -2249,8 +2337,9 @@
           <t>Hiper-reflexia</t>
         </is>
       </c>
-      <c r="H43" s="4" t="inlineStr"/>
+      <c r="H43" s="9" t="inlineStr"/>
       <c r="I43" s="4" t="inlineStr"/>
+      <c r="J43" s="4" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" s="3" t="inlineStr">
@@ -2280,8 +2369,9 @@
           <t>Autismo</t>
         </is>
       </c>
-      <c r="H44" s="4" t="inlineStr"/>
+      <c r="H44" s="9" t="inlineStr"/>
       <c r="I44" s="4" t="inlineStr"/>
+      <c r="J44" s="4" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" s="3" t="inlineStr">
@@ -2315,8 +2405,9 @@
           <t>Comportamento agressivo</t>
         </is>
       </c>
-      <c r="H45" s="4" t="inlineStr"/>
+      <c r="H45" s="9" t="inlineStr"/>
       <c r="I45" s="4" t="inlineStr"/>
+      <c r="J45" s="4" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" s="3" t="inlineStr">
@@ -2350,8 +2441,9 @@
           <t>Retrusão do terço médio da face</t>
         </is>
       </c>
-      <c r="H46" s="4" t="inlineStr"/>
+      <c r="H46" s="9" t="inlineStr"/>
       <c r="I46" s="4" t="inlineStr"/>
+      <c r="J46" s="4" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" s="3" t="inlineStr">
@@ -2385,8 +2477,9 @@
           <t>Distúrbio da marcha</t>
         </is>
       </c>
-      <c r="H47" s="4" t="inlineStr"/>
+      <c r="H47" s="9" t="inlineStr"/>
       <c r="I47" s="4" t="inlineStr"/>
+      <c r="J47" s="4" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" s="3" t="inlineStr">
@@ -2420,8 +2513,9 @@
           <t>Braquidactilia</t>
         </is>
       </c>
-      <c r="H48" s="4" t="inlineStr"/>
+      <c r="H48" s="9" t="inlineStr"/>
       <c r="I48" s="4" t="inlineStr"/>
+      <c r="J48" s="4" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" s="3" t="inlineStr">
@@ -2455,8 +2549,9 @@
           <t>Atrofia cerebral</t>
         </is>
       </c>
-      <c r="H49" s="4" t="inlineStr"/>
+      <c r="H49" s="9" t="inlineStr"/>
       <c r="I49" s="4" t="inlineStr"/>
+      <c r="J49" s="4" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" s="3" t="inlineStr">
@@ -2490,8 +2585,13 @@
           <t>Concentração circulante de lactato aumentada</t>
         </is>
       </c>
-      <c r="H50" s="4" t="inlineStr"/>
+      <c r="H50" s="9" t="inlineStr">
+        <is>
+          <t>Forma do rótulo: dos 129 rótulos oficiais do tipo 'Increased/Decreased/Abnormal circulating ... concentration', 'Hiper-/Hipo-' aparece em 0; a forma é descritiva (ex.: HP:0002920, 'Concentração de ACTH circulante diminuída'). Em inglês, 'Hyperlactatemia' não é sinônimo nesta versão do HPO. Se 'Hiperlactatemia' for o termo usual, indique-o em reviewer_notes como sinônimo.</t>
+        </is>
+      </c>
       <c r="I50" s="4" t="inlineStr"/>
+      <c r="J50" s="4" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" s="3" t="inlineStr">
@@ -2525,11 +2625,16 @@
           <t>Anormalidade da mão</t>
         </is>
       </c>
-      <c r="H51" s="4" t="inlineStr"/>
+      <c r="H51" s="9" t="inlineStr">
+        <is>
+          <t>Padronização: a tradução oficial do HPO usa 'Anomalia', não 'Anormalidade'. 264 rótulos oficiais começam com 'Anomalia' e 0 com 'Anormalidade'; dos 201 termos 'Abnormality of ...' já traduzidos, 200 começam com 'Anomalia' (ex.: HP:0000002, 'Anomalia da altura corporal').</t>
+        </is>
+      </c>
       <c r="I51" s="4" t="inlineStr"/>
+      <c r="J51" s="4" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I51"/>
+  <autoFilter ref="A1:J51"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>

</xml_diff>